<commit_message>
Completed Content for Checkpoint 2
Completed Report and Tests as well as Designs for Checkpoint 2 that was due 11 September 2026
</commit_message>
<xml_diff>
--- a/MCTR/Juan_Fourie/Gearbox_Design/Motor_Gearbox_Drum_Calculations.xlsx
+++ b/MCTR/Juan_Fourie/Gearbox_Design/Motor_Gearbox_Drum_Calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NoordWes Universiteit\Mechatronics Engineering\Jaar 3\Semester 2\MCTR327\Eng_DesignProject_GantryCrane_Group-18\MCTR\Juan_Fourie\Gearbox_Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8288C71-F6BD-45B0-86C5-CBE99B6B1353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A432642-88F0-42B6-9E1B-9AB7C7756A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B04408CB-7577-4945-9BAD-2F544BAEE8BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B04408CB-7577-4945-9BAD-2F544BAEE8BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,43 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Addendum_Circle">Sheet1!$C$7</definedName>
-    <definedName name="Base_Circle">Sheet1!$C$10</definedName>
-    <definedName name="Clearance_Circle">Sheet1!$C$9</definedName>
-    <definedName name="Module">Sheet1!$C$3</definedName>
-    <definedName name="Number_of_Teeth">Sheet1!$C$4</definedName>
-    <definedName name="Pitch_Circle">Sheet1!$C$6</definedName>
-    <definedName name="Pressure_Angle">Sheet1!$C$5</definedName>
-    <definedName name="Root_Circle">Sheet1!$C$8</definedName>
+    <definedName name="Addendum_Circle">Sheet1!$C$21</definedName>
+    <definedName name="Base_Circle">Sheet1!$C$24</definedName>
+    <definedName name="Clearance_Circle">Sheet1!$C$23</definedName>
+    <definedName name="Drum_Circumference">Sheet1!$C$40</definedName>
+    <definedName name="Drum_Diameter">Sheet1!$C$37</definedName>
+    <definedName name="Drum_Height">Sheet1!$C$38</definedName>
+    <definedName name="Drum_RopeLengthin1Layer">Sheet1!$C$42</definedName>
+    <definedName name="Drum_RPM">Sheet1!$C$43</definedName>
+    <definedName name="Drum_StartingSercingFactor">Sheet1!$C$39</definedName>
+    <definedName name="Drum_StartingServingFactor">Sheet1!$C$39</definedName>
+    <definedName name="DrumLoopsinCirc">Sheet1!$C$41</definedName>
+    <definedName name="Largest_Gear_Teeth">Sheet1!$C$28</definedName>
+    <definedName name="Line_Speed">Sheet1!$C$36</definedName>
+    <definedName name="Max_Load">Sheet1!$C$2</definedName>
+    <definedName name="Module">Sheet1!$C$16</definedName>
+    <definedName name="Motor_Mass">Sheet1!$C$58</definedName>
+    <definedName name="Motor_Power">Sheet1!$C$56</definedName>
+    <definedName name="Motor_ShaftDiameter">Sheet1!$C$59</definedName>
+    <definedName name="Motor_Speed">Sheet1!$C$57</definedName>
+    <definedName name="Motor_Torque">Sheet1!$C$61</definedName>
+    <definedName name="MotorTorque">Sheet1!$C$61</definedName>
+    <definedName name="Number_of_Teeth">Sheet1!$C$17</definedName>
+    <definedName name="PerStageWork">Sheet1!$C$26</definedName>
+    <definedName name="Pitch_Circle">Sheet1!$C$20</definedName>
+    <definedName name="Pressure_Angle">Sheet1!$C$18</definedName>
+    <definedName name="Reduction_Ratio">Sheet1!$C$25</definedName>
+    <definedName name="Root_Circle">Sheet1!$C$22</definedName>
+    <definedName name="Rope_Diameter">Sheet1!$C$49</definedName>
+    <definedName name="Rope_Length">Sheet1!$C$50</definedName>
+    <definedName name="Rope_Wraps">Sheet1!$C$51</definedName>
+    <definedName name="Sheet_Height">Sheet1!$C$10</definedName>
+    <definedName name="Sheet_Length">Sheet1!$C$11</definedName>
+    <definedName name="Sheet_Width">Sheet1!$C$9</definedName>
+    <definedName name="small_to_large_ratio">Sheet1!$B$29</definedName>
+    <definedName name="Smallest_Gear_Teeth">Sheet1!$C$27</definedName>
+    <definedName name="Stroke">Sheet1!$C$3</definedName>
+    <definedName name="Stroke_Speed">Sheet1!$C$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,8 +79,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
   <si>
     <t>Max Load</t>
   </si>
@@ -59,15 +110,9 @@
     <t>kg</t>
   </si>
   <si>
-    <t>Drum Dia</t>
-  </si>
-  <si>
     <t>mm</t>
   </si>
   <si>
-    <t>Motor RPM</t>
-  </si>
-  <si>
     <t>rpm</t>
   </si>
   <si>
@@ -225,13 +270,22 @@
   </si>
   <si>
     <t>Ng</t>
+  </si>
+  <si>
+    <t>Design Main Specifications</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,6 +297,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -262,7 +324,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -270,11 +332,478 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC00000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC00000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC00000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC00000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC00000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -282,10 +811,58 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -322,7 +899,7 @@
       <xdr:col>41</xdr:col>
       <xdr:colOff>402596</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>95506</xdr:rowOff>
+      <xdr:rowOff>21211</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -355,67 +932,23 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>302895</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>40005</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>40</xdr:col>
-      <xdr:colOff>364464</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>168082</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{735F9A7E-F9E3-5975-C5F5-8D900AC995AB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19400520" y="3028950"/>
-          <a:ext cx="7031964" cy="5098222"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>36195</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="9" name="Rectangle 8">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB893FF9-3263-8DCD-D7AF-EF361F58B35F}"/>
@@ -426,8 +959,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="645795" y="5257800"/>
-          <a:ext cx="1268730" cy="609600"/>
+          <a:off x="9500235" y="7720965"/>
+          <a:ext cx="1268730" cy="615315"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -494,24 +1027,24 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>434340</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>601980</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>491490</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>59055</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>49530</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>112395</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Rectangle 10">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        <xdr:cNvPr id="5" name="Rectangle 4">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A785D5F5-73C7-4B40-BFAA-AC4927C3CAFE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52E81FCC-DEDC-D7D7-CB2F-1FB052950F5E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -519,8 +1052,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2225040" y="5234940"/>
-          <a:ext cx="1276350" cy="615315"/>
+          <a:off x="11018520" y="7719060"/>
+          <a:ext cx="1276350" cy="622935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1321,472 +1854,533 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7090C4EA-807B-4A95-883D-8A7A770966AE}">
-  <dimension ref="B1:Z28"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+    </row>
+    <row r="2" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="32">
+        <v>30</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="23">
+        <v>1600</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="6"/>
+      <c r="C4" s="24">
+        <v>80</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+    </row>
+    <row r="9" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29">
+        <v>600</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="25">
+        <v>3</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="30">
+        <v>400</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+    </row>
+    <row r="15" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="8">
+        <v>2</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17">
+        <v>30</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="8">
+        <v>25</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="10">
+        <v>15</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="12">
+        <f>Module*Number_of_Teeth</f>
+        <v>60</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21">
+        <f>Pitch_Circle+(2*Module)</f>
+        <v>64</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <f>Pitch_Circle-(2*(1.25*Module))</f>
+        <v>55</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23">
+        <f>Pitch_Circle-Module*2</f>
+        <v>56</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="17">
+        <f>Pitch_Circle*COS(RADIANS(Pressure_Angle))</f>
+        <v>54.378467222198999</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="13">
+        <f>Motor_Speed/Drum_RPM</f>
+        <v>44.505895925855405</v>
+      </c>
+      <c r="E25" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="15" cm="1">
+        <f t="array" ref="C26">SQRT(Reduction_Ratio)</f>
+        <v>6.6712739357528559</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="15">
+        <f>_xlfn.CEILING.MATH((2/((1+2*PerStageWork)*SIN(RADIANS(Pressure_Angle))^2))*(PerStageWork+SQRT(PerStageWork^2+(1+2*PerStageWork)*SIN(RADIANS(Pressure_Angle))^2)))</f>
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="15">
+        <f>_xlfn.CEILING.MATH((C27^2*SIN(RADIANS(Pressure_Angle))^2-4*1^2)/(4*1-2*C27*SIN(RADIANS(Pressure_Angle))^2))</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="47"/>
+      <c r="B29" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="46">
+        <f>Largest_Gear_Teeth/Smallest_Gear_Teeth</f>
+        <v>22.727272727272727</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="44"/>
+    </row>
+    <row r="35" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+    </row>
+    <row r="36" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="22">
+        <v>88</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="25">
+        <v>50</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="25">
+        <v>60</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C39" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="D39" s="21"/>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B40" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40">
+        <f>Drum_Diameter*PI()</f>
+        <v>157.07963267948966</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B41" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="3"/>
-    </row>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3">
+      <c r="C41">
+        <f>Drum_Height/Rope_Diameter</f>
+        <v>12</v>
+      </c>
+      <c r="D41" s="15"/>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B42" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42">
+        <f>DrumLoopsinCirc*Drum_Circumference</f>
+        <v>1884.9555921538758</v>
+      </c>
+      <c r="D42" s="15"/>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B43" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43" cm="1">
+        <f t="array" ref="C43">(Stroke_Speed/1000)/(Drum_Circumference/1000)*60</f>
+        <v>30.557749073643905</v>
+      </c>
+      <c r="D43" s="15"/>
+    </row>
+    <row r="44" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B44" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" s="17" cm="1">
+        <f t="array" ref="C44">Max_Load*9.81*((Drum_Diameter/2)/1000)*Drum_StartingServingFactor</f>
+        <v>11.036250000000001</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+      <c r="E48" s="48"/>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+    </row>
+    <row r="49" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B49" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="25">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
-        <v>50</v>
-      </c>
-      <c r="K3" t="s">
-        <v>0</v>
-      </c>
-      <c r="L3">
+      <c r="D49" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B50" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C50" s="23">
+        <v>1600</v>
+      </c>
+      <c r="D50" s="20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B51" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="M3" t="s">
+      <c r="C51" s="45">
+        <f>Stroke/Drum_Circumference</f>
+        <v>10.185916357881302</v>
+      </c>
+      <c r="D51" s="46"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="I53" s="33"/>
+    </row>
+    <row r="55" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="C55" s="37"/>
+      <c r="D55" s="37"/>
+      <c r="E55" s="48"/>
+      <c r="F55" s="48"/>
+      <c r="G55" s="48"/>
+    </row>
+    <row r="56" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B56" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" s="22">
+        <v>0.18</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B57" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" s="25">
+        <v>1360</v>
+      </c>
+      <c r="D57" s="26" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B58" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="23">
+        <v>4.83</v>
+      </c>
+      <c r="D58" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="O3" t="s">
-        <v>10</v>
-      </c>
-      <c r="P3">
-        <v>600</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>50</v>
-      </c>
-      <c r="K4" t="s">
+    </row>
+    <row r="59" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B59" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C59" s="25">
+        <v>11</v>
+      </c>
+      <c r="D59" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="L4">
-        <v>70</v>
-      </c>
-      <c r="M4" t="s">
-        <v>3</v>
-      </c>
-      <c r="O4" t="s">
-        <v>11</v>
-      </c>
-      <c r="P4">
-        <v>3</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5">
+    </row>
+    <row r="60" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B60" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C60" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="22" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B61" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C61" s="39">
+        <f>Motor_Power/(Motor_Speed*2*PI()/60)*1000</f>
+        <v>1.2638774892591689</v>
+      </c>
+      <c r="D61" s="40" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" t="s">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>1360</v>
-      </c>
-      <c r="M5" t="s">
-        <v>5</v>
-      </c>
-      <c r="O5" t="s">
+      <c r="C62" s="42">
+        <f>3*Motor_Torque</f>
+        <v>3.7916324677775064</v>
+      </c>
+      <c r="D62" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="P5">
-        <v>400</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6">
-        <f>Module*Number_of_Teeth</f>
-        <v>150</v>
-      </c>
-      <c r="D6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K6" t="s">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>1600</v>
-      </c>
-      <c r="M6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7">
-        <f>Pitch_Circle+(2*Module)</f>
-        <v>160</v>
-      </c>
-      <c r="D7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>80</v>
-      </c>
-      <c r="M7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8">
-        <f>Pitch_Circle-(2*(1.25*Module))</f>
-        <v>137.5</v>
-      </c>
-      <c r="D8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9">
-        <f>Pitch_Circle-Module*2</f>
-        <v>140</v>
-      </c>
-      <c r="D9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10">
-        <f>Pitch_Circle*COS(RADIANS(Pressure_Angle))</f>
-        <v>140.95389311788625</v>
-      </c>
-      <c r="D10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14">
-        <f>V21/J26</f>
-        <v>44.505895925855405</v>
-      </c>
-      <c r="D14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15">
-        <f>SQRT(C14)</f>
-        <v>6.6712739357528559</v>
-      </c>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16">
-        <f>_xlfn.CEILING.MATH((2/((1+2*Module)*SIN(RADIANS(Pressure_Angle))^2))*(Module+SQRT(Module^2+(1+2*Module)*SIN(RADIANS(Pressure_Angle))^2)))</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17">
-        <f>_xlfn.CEILING.MATH((C16^2*SIN(RADIANS(Pressure_Angle))^2-4*1^2)/(4*1-2*C16*SIN(RADIANS(Pressure_Angle))^2))</f>
-        <v>102</v>
-      </c>
-    </row>
-    <row r="19" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="4"/>
-      <c r="U19" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="V19" s="4"/>
-      <c r="W19" s="4"/>
-      <c r="X19" s="4"/>
-      <c r="Y19" s="4"/>
-      <c r="Z19" s="4"/>
-    </row>
-    <row r="20" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I20" t="s">
-        <v>25</v>
-      </c>
-      <c r="J20">
-        <v>88</v>
-      </c>
-      <c r="K20" t="s">
-        <v>7</v>
-      </c>
-      <c r="O20" t="s">
-        <v>29</v>
-      </c>
-      <c r="P20">
-        <v>5</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>3</v>
-      </c>
-      <c r="U20" t="s">
-        <v>16</v>
-      </c>
-      <c r="V20">
-        <v>0.18</v>
-      </c>
-      <c r="W20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I21" t="s">
-        <v>28</v>
-      </c>
-      <c r="J21">
-        <f>J22*PI()</f>
-        <v>157.07963267948966</v>
-      </c>
-      <c r="K21" t="s">
-        <v>3</v>
-      </c>
-      <c r="O21" t="s">
-        <v>31</v>
-      </c>
-      <c r="P21">
-        <v>1600</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>3</v>
-      </c>
-      <c r="U21" t="s">
-        <v>17</v>
-      </c>
-      <c r="V21">
-        <v>1360</v>
-      </c>
-      <c r="W21" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I22" t="s">
-        <v>29</v>
-      </c>
-      <c r="J22">
-        <v>50</v>
-      </c>
-      <c r="K22" t="s">
-        <v>3</v>
-      </c>
-      <c r="O22" t="s">
-        <v>32</v>
-      </c>
-      <c r="P22">
-        <f>L6/J21</f>
-        <v>10.185916357881302</v>
-      </c>
-      <c r="U22" t="s">
-        <v>18</v>
-      </c>
-      <c r="V22">
-        <v>4.83</v>
-      </c>
-      <c r="W22" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I23" t="s">
-        <v>34</v>
-      </c>
-      <c r="J23">
-        <v>60</v>
-      </c>
-      <c r="K23" t="s">
-        <v>3</v>
-      </c>
-      <c r="U23" t="s">
-        <v>19</v>
-      </c>
-      <c r="V23">
-        <v>11</v>
-      </c>
-      <c r="W23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I24" t="s">
-        <v>35</v>
-      </c>
-      <c r="J24">
-        <f>J23/P20</f>
-        <v>12</v>
-      </c>
-      <c r="U24" t="s">
-        <v>20</v>
-      </c>
-      <c r="V24" t="s">
-        <v>23</v>
-      </c>
-      <c r="W24" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I25" t="s">
-        <v>36</v>
-      </c>
-      <c r="J25">
-        <f>J24*J21</f>
-        <v>1884.9555921538758</v>
-      </c>
-      <c r="U25" t="s">
-        <v>21</v>
-      </c>
-      <c r="V25">
-        <f>V20/(V21*2*PI()/60)*1000</f>
-        <v>1.2638774892591689</v>
-      </c>
-      <c r="W25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I26" t="s">
-        <v>27</v>
-      </c>
-      <c r="J26">
-        <f>(L7/1000)/(J21/1000)*60</f>
-        <v>30.557749073643905</v>
-      </c>
-      <c r="U26" t="s">
-        <v>22</v>
-      </c>
-      <c r="V26">
-        <f>3*V25</f>
-        <v>3.7916324677775064</v>
-      </c>
-      <c r="W26" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I27" t="s">
-        <v>55</v>
-      </c>
-      <c r="J27">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="I28" t="s">
-        <v>26</v>
-      </c>
-      <c r="J28">
-        <f>L3*9.81*((J22/2)/1000)*J27</f>
-        <v>11.036250000000001</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="U19:Z19"/>
-    <mergeCell ref="I19:N19"/>
-    <mergeCell ref="O19:T19"/>
-    <mergeCell ref="B1:G1"/>
+  <mergeCells count="6">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B55:D55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>